<commit_message>
docs(mailtemplate-import): .Eeg.Name and .Eeg.Description both map to eeg.name
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/test.xlsx
+++ b/database/test.xlsx
@@ -10,7 +10,7 @@
     <sheet name="ZP-List" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'ZP-List'!$A$1:$AH$10</definedName>
+    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'ZP-List'!$A$1:$I$25</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
@@ -1236,6 +1236,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$AH$10"/>
+  <autoFilter ref="$A$1:$I$25"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: CHANGELOG entry back under [Unreleased] (misplaced by the master merge), {eeg.name} wording effects, import note; test.xlsx as on master
test.xlsx was committed by accident with 048b6c3 (rewritten by excel_test.go on every run).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/test.xlsx
+++ b/database/test.xlsx
@@ -10,7 +10,7 @@
     <sheet name="ZP-List" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'ZP-List'!$A$1:$I$25</definedName>
+    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'ZP-List'!$A$1:$AH$10</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
@@ -1236,6 +1236,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$I$25"/>
+  <autoFilter ref="$A$1:$AH$10"/>
 </worksheet>
 </file>
</xml_diff>